<commit_message>
New file to deal with stage of model after basic stats analysis
</commit_message>
<xml_diff>
--- a/mfc_analysis.xlsx
+++ b/mfc_analysis.xlsx
@@ -492,7 +492,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2024-07-24</t>
+          <t>24/07/2024</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -535,7 +535,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2024-07-29</t>
+          <t>29/07/2024</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -578,7 +578,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2024-08-02</t>
+          <t>02/08/2024</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -621,7 +621,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2024-08-06</t>
+          <t>06/08/2024</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -664,7 +664,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2024-08-08</t>
+          <t>08/08/2024</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -707,7 +707,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2024-09-16</t>
+          <t>16/09/2024</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -750,7 +750,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2024-09-24</t>
+          <t>24/09/2024</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -793,7 +793,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2024-10-02</t>
+          <t>02/10/2024</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -836,7 +836,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2024-10-10</t>
+          <t>10/10/2024</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -879,7 +879,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2024-10-12</t>
+          <t>12/10/2024</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -922,7 +922,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2024-10-16</t>
+          <t>16/10/2024</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -965,7 +965,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2024-10-25</t>
+          <t>25/10/2024</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -1008,7 +1008,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2024-12-10</t>
+          <t>10/12/2024</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -1051,7 +1051,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2025-02-07</t>
+          <t>07/02/2025</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -1094,7 +1094,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2025-02-11</t>
+          <t>11/02/2025</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -1137,7 +1137,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2025-02-14</t>
+          <t>14/02/2025</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -1180,7 +1180,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2025-02-21</t>
+          <t>21/02/2025</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -1223,7 +1223,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2025-02-24</t>
+          <t>24/02/2025</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -1266,7 +1266,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2025-04-02</t>
+          <t>02/04/2025</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -1309,7 +1309,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2025-04-03</t>
+          <t>03/04/2025</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1352,7 +1352,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2025-04-04</t>
+          <t>04/04/2025</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -1395,7 +1395,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2025-04-28</t>
+          <t>28/04/2025</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1438,7 +1438,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2025-04-30</t>
+          <t>30/04/2025</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -1481,7 +1481,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2025-05-07</t>
+          <t>07/05/2025</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1524,7 +1524,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2025-05-08</t>
+          <t>08/05/2025</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -1567,7 +1567,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2025-05-09</t>
+          <t>09/05/2025</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1610,7 +1610,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2025-05-12</t>
+          <t>12/05/2025</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -1653,7 +1653,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2025-05-13</t>
+          <t>13/05/2025</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1696,7 +1696,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2025-05-18</t>
+          <t>18/05/2025</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -1820,7 +1820,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2024-07-24</t>
+          <t>24/07/2024</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -1863,7 +1863,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2024-07-29</t>
+          <t>29/07/2024</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -1906,7 +1906,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2024-08-02</t>
+          <t>02/08/2024</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -1949,7 +1949,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2024-08-06</t>
+          <t>06/08/2024</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -1992,7 +1992,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2024-08-08</t>
+          <t>08/08/2024</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -2035,7 +2035,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2024-09-16</t>
+          <t>16/09/2024</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -2078,7 +2078,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2024-09-24</t>
+          <t>24/09/2024</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -2121,7 +2121,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2024-10-02</t>
+          <t>02/10/2024</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -2164,7 +2164,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2024-10-10</t>
+          <t>10/10/2024</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -2207,7 +2207,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2024-10-12</t>
+          <t>12/10/2024</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -2250,7 +2250,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2024-10-16</t>
+          <t>16/10/2024</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -2293,7 +2293,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2024-10-25</t>
+          <t>25/10/2024</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -2336,7 +2336,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2024-12-10</t>
+          <t>10/12/2024</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -2379,7 +2379,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2025-02-07</t>
+          <t>07/02/2025</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -2422,7 +2422,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2025-02-11</t>
+          <t>11/02/2025</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -2465,7 +2465,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2025-02-14</t>
+          <t>14/02/2025</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -2508,7 +2508,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2025-02-21</t>
+          <t>21/02/2025</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -2551,7 +2551,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2025-02-24</t>
+          <t>24/02/2025</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -2594,7 +2594,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2025-04-02</t>
+          <t>02/04/2025</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -2637,7 +2637,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2025-04-03</t>
+          <t>03/04/2025</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -2680,7 +2680,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2025-04-04</t>
+          <t>04/04/2025</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -2723,7 +2723,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2025-04-28</t>
+          <t>28/04/2025</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -2766,7 +2766,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2025-04-30</t>
+          <t>30/04/2025</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -2809,7 +2809,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2025-05-07</t>
+          <t>07/05/2025</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -2852,7 +2852,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2025-05-08</t>
+          <t>08/05/2025</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -2895,7 +2895,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2025-05-09</t>
+          <t>09/05/2025</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -2938,7 +2938,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2025-05-12</t>
+          <t>12/05/2025</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -2981,7 +2981,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2025-05-13</t>
+          <t>13/05/2025</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -3024,7 +3024,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2025-05-18</t>
+          <t>18/05/2025</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -3148,7 +3148,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2024-07-24</t>
+          <t>24/07/2024</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -3191,7 +3191,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2024-07-29</t>
+          <t>29/07/2024</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -3234,7 +3234,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2024-08-02</t>
+          <t>02/08/2024</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -3277,7 +3277,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2024-08-06</t>
+          <t>06/08/2024</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -3318,7 +3318,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2024-08-08</t>
+          <t>08/08/2024</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -3361,7 +3361,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2024-09-16</t>
+          <t>16/09/2024</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -3404,7 +3404,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2024-09-24</t>
+          <t>24/09/2024</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -3447,7 +3447,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2024-10-02</t>
+          <t>02/10/2024</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -3490,7 +3490,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2024-10-10</t>
+          <t>10/10/2024</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -3533,7 +3533,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2024-10-12</t>
+          <t>12/10/2024</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -3576,7 +3576,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2024-10-16</t>
+          <t>16/10/2024</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -3619,7 +3619,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2024-10-25</t>
+          <t>25/10/2024</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -3662,7 +3662,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2024-12-10</t>
+          <t>10/12/2024</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -3705,7 +3705,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2025-02-07</t>
+          <t>07/02/2025</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -3746,7 +3746,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2025-02-11</t>
+          <t>11/02/2025</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -3789,7 +3789,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2025-02-14</t>
+          <t>14/02/2025</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -3832,7 +3832,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2025-02-21</t>
+          <t>21/02/2025</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -3875,7 +3875,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2025-02-24</t>
+          <t>24/02/2025</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -3918,7 +3918,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2025-04-02</t>
+          <t>02/04/2025</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -3961,7 +3961,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2025-04-03</t>
+          <t>03/04/2025</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -4004,7 +4004,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2025-04-04</t>
+          <t>04/04/2025</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -4047,7 +4047,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2025-04-28</t>
+          <t>28/04/2025</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -4090,7 +4090,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2025-04-30</t>
+          <t>30/04/2025</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -4133,7 +4133,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2025-05-07</t>
+          <t>07/05/2025</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -4176,7 +4176,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2025-05-08</t>
+          <t>08/05/2025</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -4219,7 +4219,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2025-05-09</t>
+          <t>09/05/2025</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -4262,7 +4262,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2025-05-12</t>
+          <t>12/05/2025</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -4305,7 +4305,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2025-05-13</t>
+          <t>13/05/2025</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -4348,7 +4348,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2025-05-18</t>
+          <t>18/05/2025</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -4472,7 +4472,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2024-07-24</t>
+          <t>24/07/2024</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -4515,7 +4515,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2024-07-29</t>
+          <t>29/07/2024</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -4558,7 +4558,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2024-08-02</t>
+          <t>02/08/2024</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -4601,7 +4601,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2024-08-06</t>
+          <t>06/08/2024</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -4642,7 +4642,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2024-08-08</t>
+          <t>08/08/2024</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -4685,7 +4685,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2024-09-16</t>
+          <t>16/09/2024</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -4728,7 +4728,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2024-09-24</t>
+          <t>24/09/2024</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -4771,7 +4771,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2024-10-02</t>
+          <t>02/10/2024</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -4814,7 +4814,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2024-10-10</t>
+          <t>10/10/2024</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -4857,7 +4857,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2024-10-12</t>
+          <t>12/10/2024</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -4900,7 +4900,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2024-10-16</t>
+          <t>16/10/2024</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -4943,7 +4943,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2024-10-25</t>
+          <t>25/10/2024</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -4986,7 +4986,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2024-12-10</t>
+          <t>10/12/2024</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -5029,7 +5029,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2025-02-07</t>
+          <t>07/02/2025</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -5070,7 +5070,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2025-02-11</t>
+          <t>11/02/2025</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -5113,7 +5113,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2025-02-14</t>
+          <t>14/02/2025</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -5156,7 +5156,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2025-02-21</t>
+          <t>21/02/2025</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -5199,7 +5199,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2025-02-24</t>
+          <t>24/02/2025</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -5242,7 +5242,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2025-04-02</t>
+          <t>02/04/2025</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -5285,7 +5285,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2025-04-03</t>
+          <t>03/04/2025</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -5328,7 +5328,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2025-04-04</t>
+          <t>04/04/2025</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -5371,7 +5371,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2025-04-28</t>
+          <t>28/04/2025</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -5414,7 +5414,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2025-04-30</t>
+          <t>30/04/2025</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -5457,7 +5457,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2025-05-07</t>
+          <t>07/05/2025</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -5500,7 +5500,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2025-05-08</t>
+          <t>08/05/2025</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -5543,7 +5543,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2025-05-09</t>
+          <t>09/05/2025</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -5586,7 +5586,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2025-05-12</t>
+          <t>12/05/2025</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -5629,7 +5629,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2025-05-13</t>
+          <t>13/05/2025</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -5672,7 +5672,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2025-05-18</t>
+          <t>18/05/2025</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -5796,7 +5796,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2024-07-24</t>
+          <t>24/07/2024</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -5839,7 +5839,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2024-07-29</t>
+          <t>29/07/2024</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -5882,7 +5882,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2024-08-02</t>
+          <t>02/08/2024</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -5925,7 +5925,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2024-08-06</t>
+          <t>06/08/2024</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -5966,7 +5966,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2024-08-08</t>
+          <t>08/08/2024</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -6009,7 +6009,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2024-09-16</t>
+          <t>16/09/2024</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -6052,7 +6052,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2024-09-24</t>
+          <t>24/09/2024</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -6095,7 +6095,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2024-10-02</t>
+          <t>02/10/2024</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -6138,7 +6138,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2024-10-10</t>
+          <t>10/10/2024</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -6181,7 +6181,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2024-10-12</t>
+          <t>12/10/2024</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -6224,7 +6224,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2024-10-16</t>
+          <t>16/10/2024</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -6267,7 +6267,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2024-10-25</t>
+          <t>25/10/2024</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -6310,7 +6310,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2024-12-10</t>
+          <t>10/12/2024</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -6353,7 +6353,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2025-02-07</t>
+          <t>07/02/2025</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -6394,7 +6394,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2025-02-11</t>
+          <t>11/02/2025</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -6437,7 +6437,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2025-02-14</t>
+          <t>14/02/2025</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -6480,7 +6480,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2025-02-21</t>
+          <t>21/02/2025</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -6523,7 +6523,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2025-02-24</t>
+          <t>24/02/2025</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -6566,7 +6566,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2025-04-02</t>
+          <t>02/04/2025</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -6609,7 +6609,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2025-04-03</t>
+          <t>03/04/2025</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -6652,7 +6652,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2025-04-04</t>
+          <t>04/04/2025</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -6695,7 +6695,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2025-04-28</t>
+          <t>28/04/2025</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -6738,7 +6738,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2025-04-30</t>
+          <t>30/04/2025</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -6781,7 +6781,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2025-05-07</t>
+          <t>07/05/2025</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -6824,7 +6824,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2025-05-08</t>
+          <t>08/05/2025</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -6867,7 +6867,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2025-05-09</t>
+          <t>09/05/2025</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -6910,7 +6910,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2025-05-12</t>
+          <t>12/05/2025</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -6953,7 +6953,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2025-05-13</t>
+          <t>13/05/2025</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -6996,7 +6996,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2025-05-18</t>
+          <t>18/05/2025</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -7120,7 +7120,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2024-07-24</t>
+          <t>24/07/2024</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -7163,7 +7163,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2024-07-29</t>
+          <t>29/07/2024</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -7206,7 +7206,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2024-08-02</t>
+          <t>02/08/2024</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -7247,7 +7247,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2024-08-06</t>
+          <t>06/08/2024</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -7288,7 +7288,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2024-08-08</t>
+          <t>08/08/2024</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -7331,7 +7331,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2024-09-16</t>
+          <t>16/09/2024</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -7374,7 +7374,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2024-09-24</t>
+          <t>24/09/2024</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -7415,7 +7415,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2024-10-02</t>
+          <t>02/10/2024</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -7458,7 +7458,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2024-10-10</t>
+          <t>10/10/2024</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -7501,7 +7501,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2024-10-12</t>
+          <t>12/10/2024</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -7544,7 +7544,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2024-10-16</t>
+          <t>16/10/2024</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -7587,7 +7587,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2024-10-25</t>
+          <t>25/10/2024</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -7630,7 +7630,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2024-12-10</t>
+          <t>10/12/2024</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -7673,7 +7673,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2025-02-07</t>
+          <t>07/02/2025</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -7714,7 +7714,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2025-02-11</t>
+          <t>11/02/2025</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -7757,7 +7757,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2025-02-14</t>
+          <t>14/02/2025</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -7800,7 +7800,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2025-02-21</t>
+          <t>21/02/2025</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -7843,7 +7843,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2025-02-24</t>
+          <t>24/02/2025</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -7886,7 +7886,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2025-04-02</t>
+          <t>02/04/2025</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -7929,7 +7929,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2025-04-03</t>
+          <t>03/04/2025</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -7972,7 +7972,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2025-04-04</t>
+          <t>04/04/2025</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -8015,7 +8015,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2025-04-28</t>
+          <t>28/04/2025</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -8058,7 +8058,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2025-04-30</t>
+          <t>30/04/2025</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -8101,7 +8101,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2025-05-07</t>
+          <t>07/05/2025</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -8144,7 +8144,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2025-05-08</t>
+          <t>08/05/2025</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -8187,7 +8187,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2025-05-09</t>
+          <t>09/05/2025</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -8230,7 +8230,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2025-05-12</t>
+          <t>12/05/2025</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -8271,7 +8271,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2025-05-13</t>
+          <t>13/05/2025</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -8314,7 +8314,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2025-05-18</t>
+          <t>18/05/2025</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -8438,7 +8438,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2024-07-24</t>
+          <t>24/07/2024</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -8481,7 +8481,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2024-07-29</t>
+          <t>29/07/2024</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -8524,7 +8524,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2024-08-02</t>
+          <t>02/08/2024</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -8567,7 +8567,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2024-08-06</t>
+          <t>06/08/2024</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -8610,7 +8610,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2024-08-08</t>
+          <t>08/08/2024</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -8653,7 +8653,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2024-09-16</t>
+          <t>16/09/2024</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -8696,7 +8696,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2024-09-24</t>
+          <t>24/09/2024</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -8739,7 +8739,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2024-10-02</t>
+          <t>02/10/2024</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -8782,7 +8782,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2024-10-10</t>
+          <t>10/10/2024</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -8825,7 +8825,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2024-10-12</t>
+          <t>12/10/2024</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -8868,7 +8868,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2024-10-16</t>
+          <t>16/10/2024</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -8911,7 +8911,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2024-10-25</t>
+          <t>25/10/2024</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -8954,7 +8954,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2024-12-10</t>
+          <t>10/12/2024</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -8997,7 +8997,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2025-02-07</t>
+          <t>07/02/2025</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -9040,7 +9040,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2025-02-11</t>
+          <t>11/02/2025</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -9083,7 +9083,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2025-02-14</t>
+          <t>14/02/2025</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -9126,7 +9126,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2025-02-21</t>
+          <t>21/02/2025</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -9169,7 +9169,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2025-02-24</t>
+          <t>24/02/2025</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -9212,7 +9212,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2025-04-02</t>
+          <t>02/04/2025</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -9255,7 +9255,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2025-04-03</t>
+          <t>03/04/2025</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -9298,7 +9298,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2025-04-04</t>
+          <t>04/04/2025</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -9341,7 +9341,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2025-04-28</t>
+          <t>28/04/2025</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -9384,7 +9384,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2025-04-30</t>
+          <t>30/04/2025</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -9427,7 +9427,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2025-05-07</t>
+          <t>07/05/2025</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -9470,7 +9470,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2025-05-08</t>
+          <t>08/05/2025</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -9513,7 +9513,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2025-05-09</t>
+          <t>09/05/2025</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -9556,7 +9556,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2025-05-12</t>
+          <t>12/05/2025</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -9599,7 +9599,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2025-05-13</t>
+          <t>13/05/2025</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -9642,7 +9642,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2025-05-18</t>
+          <t>18/05/2025</t>
         </is>
       </c>
       <c r="B30" t="n">

</xml_diff>